<commit_message>
cambio en web hsn y cambio en diseño correo
</commit_message>
<xml_diff>
--- a/data/precios_creatina.xlsx
+++ b/data/precios_creatina.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F197"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5539,7 +5539,7 @@
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
-        <v>45987.42764274263</v>
+        <v>45987.42764274305</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -5556,8 +5556,112 @@
           <t>10,90€</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
+      <c r="E197" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F197" s="3" t="n">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46144.565589375</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>CREATINA MONOHIDRATO EN POLVO (200 MESH)</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>22,50 €</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F198" s="3" t="n">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46144.56702692129</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>CREATINA MONOHIDRATO EN POLVO (200 MESH)</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>22,50 €</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F199" s="3" t="n">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46144.58307390046</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>CREATINA MONOHIDRATO EN POLVO (200 MESH)</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>22,50 €</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F200" s="3" t="n">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46144.71269611372</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>CREATINA MONOHIDRATO EN POLVO (200 MESH)</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>22,50 €</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Añade actualización manual, recordatorios y productos
</commit_message>
<xml_diff>
--- a/data/precios_creatina.xlsx
+++ b/data/precios_creatina.xlsx
@@ -16,11 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -60,13 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +486,7 @@
       <c r="E2" t="n">
         <v>12.88</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>45804</v>
       </c>
     </row>
@@ -515,7 +512,7 @@
       <c r="E3" t="n">
         <v>12.88</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="2" t="n">
         <v>45804</v>
       </c>
     </row>
@@ -541,7 +538,7 @@
       <c r="E4" t="n">
         <v>15.41</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>45805</v>
       </c>
     </row>
@@ -567,7 +564,7 @@
       <c r="E5" t="n">
         <v>12.88</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="2" t="n">
         <v>45806</v>
       </c>
     </row>
@@ -593,7 +590,7 @@
       <c r="E6" t="n">
         <v>12.88</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="2" t="n">
         <v>45806</v>
       </c>
     </row>
@@ -619,7 +616,7 @@
       <c r="E7" t="n">
         <v>15.41</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="2" t="n">
         <v>45807</v>
       </c>
     </row>
@@ -645,7 +642,7 @@
       <c r="E8" t="n">
         <v>15.41</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>45808</v>
       </c>
     </row>
@@ -671,7 +668,7 @@
       <c r="E9" t="n">
         <v>15.41</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="2" t="n">
         <v>45809</v>
       </c>
     </row>
@@ -697,7 +694,7 @@
       <c r="E10" t="n">
         <v>15.41</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="2" t="n">
         <v>45810</v>
       </c>
     </row>
@@ -723,7 +720,7 @@
       <c r="E11" t="n">
         <v>15.41</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="2" t="n">
         <v>45811</v>
       </c>
     </row>
@@ -749,7 +746,7 @@
       <c r="E12" t="n">
         <v>12.88</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="2" t="n">
         <v>45812</v>
       </c>
     </row>
@@ -775,7 +772,7 @@
       <c r="E13" t="n">
         <v>15.41</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="2" t="n">
         <v>45813</v>
       </c>
     </row>
@@ -801,7 +798,7 @@
       <c r="E14" t="n">
         <v>15.41</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="2" t="n">
         <v>45814</v>
       </c>
     </row>
@@ -827,7 +824,7 @@
       <c r="E15" t="n">
         <v>15.41</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="2" t="n">
         <v>45815</v>
       </c>
     </row>
@@ -853,7 +850,7 @@
       <c r="E16" t="n">
         <v>15.41</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="2" t="n">
         <v>45816</v>
       </c>
     </row>
@@ -879,7 +876,7 @@
       <c r="E17" t="n">
         <v>15.41</v>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="2" t="n">
         <v>45817</v>
       </c>
     </row>
@@ -905,7 +902,7 @@
       <c r="E18" t="n">
         <v>15.41</v>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="2" t="n">
         <v>45818</v>
       </c>
     </row>
@@ -931,7 +928,7 @@
       <c r="E19" t="n">
         <v>15.41</v>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -957,7 +954,7 @@
       <c r="E20" t="n">
         <v>15.41</v>
       </c>
-      <c r="F20" s="3" t="n">
+      <c r="F20" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -983,7 +980,7 @@
       <c r="E21" t="n">
         <v>15.41</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1009,7 +1006,7 @@
       <c r="E22" t="n">
         <v>15.41</v>
       </c>
-      <c r="F22" s="3" t="n">
+      <c r="F22" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1035,7 +1032,7 @@
       <c r="E23" t="n">
         <v>15.41</v>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1061,7 +1058,7 @@
       <c r="E24" t="n">
         <v>15.41</v>
       </c>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1087,7 +1084,7 @@
       <c r="E25" t="n">
         <v>15.41</v>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1113,7 +1110,7 @@
       <c r="E26" t="n">
         <v>15.41</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1139,7 +1136,7 @@
       <c r="E27" t="n">
         <v>15.41</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1165,7 +1162,7 @@
       <c r="E28" t="n">
         <v>15.41</v>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1191,7 +1188,7 @@
       <c r="E29" t="n">
         <v>15.41</v>
       </c>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1217,7 +1214,7 @@
       <c r="E30" t="n">
         <v>15.41</v>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1243,7 +1240,7 @@
       <c r="E31" t="n">
         <v>15.41</v>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1269,7 +1266,7 @@
       <c r="E32" t="n">
         <v>15.41</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1295,7 +1292,7 @@
       <c r="E33" t="n">
         <v>15.41</v>
       </c>
-      <c r="F33" s="3" t="n">
+      <c r="F33" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1321,7 +1318,7 @@
       <c r="E34" t="n">
         <v>15.41</v>
       </c>
-      <c r="F34" s="3" t="n">
+      <c r="F34" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1347,7 +1344,7 @@
       <c r="E35" t="n">
         <v>15.41</v>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1373,7 +1370,7 @@
       <c r="E36" t="n">
         <v>15.41</v>
       </c>
-      <c r="F36" s="3" t="n">
+      <c r="F36" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1399,7 +1396,7 @@
       <c r="E37" t="n">
         <v>15.41</v>
       </c>
-      <c r="F37" s="3" t="n">
+      <c r="F37" s="2" t="n">
         <v>45833</v>
       </c>
     </row>
@@ -1425,7 +1422,7 @@
       <c r="E38" t="n">
         <v>12.88</v>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="2" t="n">
         <v>45834</v>
       </c>
     </row>
@@ -1451,7 +1448,7 @@
       <c r="E39" t="n">
         <v>15.41</v>
       </c>
-      <c r="F39" s="3" t="n">
+      <c r="F39" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1477,7 +1474,7 @@
       <c r="E40" t="n">
         <v>15.41</v>
       </c>
-      <c r="F40" s="3" t="n">
+      <c r="F40" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1503,7 +1500,7 @@
       <c r="E41" t="n">
         <v>15.41</v>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1529,7 +1526,7 @@
       <c r="E42" t="n">
         <v>15.41</v>
       </c>
-      <c r="F42" s="3" t="n">
+      <c r="F42" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1555,7 +1552,7 @@
       <c r="E43" t="n">
         <v>15.41</v>
       </c>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1581,7 +1578,7 @@
       <c r="E44" t="n">
         <v>15.41</v>
       </c>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1607,7 +1604,7 @@
       <c r="E45" t="n">
         <v>15.41</v>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1633,7 +1630,7 @@
       <c r="E46" t="n">
         <v>15.41</v>
       </c>
-      <c r="F46" s="3" t="n">
+      <c r="F46" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1659,7 +1656,7 @@
       <c r="E47" t="n">
         <v>15.41</v>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F47" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1685,7 +1682,7 @@
       <c r="E48" t="n">
         <v>15.41</v>
       </c>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1711,7 +1708,7 @@
       <c r="E49" t="n">
         <v>15.41</v>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F49" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1737,7 +1734,7 @@
       <c r="E50" t="n">
         <v>15.41</v>
       </c>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1763,7 +1760,7 @@
       <c r="E51" t="n">
         <v>15.41</v>
       </c>
-      <c r="F51" s="3" t="n">
+      <c r="F51" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1789,7 +1786,7 @@
       <c r="E52" t="n">
         <v>15.41</v>
       </c>
-      <c r="F52" s="3" t="n">
+      <c r="F52" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1815,7 +1812,7 @@
       <c r="E53" t="n">
         <v>15.41</v>
       </c>
-      <c r="F53" s="3" t="n">
+      <c r="F53" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1841,7 +1838,7 @@
       <c r="E54" t="n">
         <v>15.41</v>
       </c>
-      <c r="F54" s="3" t="n">
+      <c r="F54" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1867,7 +1864,7 @@
       <c r="E55" t="n">
         <v>15.41</v>
       </c>
-      <c r="F55" s="3" t="n">
+      <c r="F55" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1893,7 +1890,7 @@
       <c r="E56" t="n">
         <v>15.41</v>
       </c>
-      <c r="F56" s="3" t="n">
+      <c r="F56" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1919,7 +1916,7 @@
       <c r="E57" t="n">
         <v>15.41</v>
       </c>
-      <c r="F57" s="3" t="n">
+      <c r="F57" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1945,7 +1942,7 @@
       <c r="E58" t="n">
         <v>15.41</v>
       </c>
-      <c r="F58" s="3" t="n">
+      <c r="F58" s="2" t="n">
         <v>45853</v>
       </c>
     </row>
@@ -1971,7 +1968,7 @@
       <c r="E59" t="n">
         <v>15.41</v>
       </c>
-      <c r="F59" s="3" t="n">
+      <c r="F59" s="2" t="n">
         <v>45854</v>
       </c>
     </row>
@@ -1997,7 +1994,7 @@
       <c r="E60" t="n">
         <v>15.41</v>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="F60" s="2" t="n">
         <v>45854</v>
       </c>
     </row>
@@ -2023,7 +2020,7 @@
       <c r="E61" t="n">
         <v>12.88</v>
       </c>
-      <c r="F61" s="3" t="n">
+      <c r="F61" s="2" t="n">
         <v>45855</v>
       </c>
     </row>
@@ -2049,7 +2046,7 @@
       <c r="E62" t="n">
         <v>12.88</v>
       </c>
-      <c r="F62" s="3" t="n">
+      <c r="F62" s="2" t="n">
         <v>45855</v>
       </c>
     </row>
@@ -2075,7 +2072,7 @@
       <c r="E63" t="n">
         <v>12.88</v>
       </c>
-      <c r="F63" s="3" t="n">
+      <c r="F63" s="2" t="n">
         <v>45856</v>
       </c>
     </row>
@@ -2101,7 +2098,7 @@
       <c r="E64" t="n">
         <v>15.41</v>
       </c>
-      <c r="F64" s="3" t="n">
+      <c r="F64" s="2" t="n">
         <v>45857</v>
       </c>
     </row>
@@ -2127,7 +2124,7 @@
       <c r="E65" t="n">
         <v>15.41</v>
       </c>
-      <c r="F65" s="3" t="n">
+      <c r="F65" s="2" t="n">
         <v>45858</v>
       </c>
     </row>
@@ -2153,7 +2150,7 @@
       <c r="E66" t="n">
         <v>15.41</v>
       </c>
-      <c r="F66" s="3" t="n">
+      <c r="F66" s="2" t="n">
         <v>45859</v>
       </c>
     </row>
@@ -2179,7 +2176,7 @@
       <c r="E67" t="n">
         <v>15.41</v>
       </c>
-      <c r="F67" s="3" t="n">
+      <c r="F67" s="2" t="n">
         <v>45860</v>
       </c>
     </row>
@@ -2205,7 +2202,7 @@
       <c r="E68" t="n">
         <v>12.88</v>
       </c>
-      <c r="F68" s="3" t="n">
+      <c r="F68" s="2" t="n">
         <v>45861</v>
       </c>
     </row>
@@ -2231,7 +2228,7 @@
       <c r="E69" t="n">
         <v>15.41</v>
       </c>
-      <c r="F69" s="3" t="n">
+      <c r="F69" s="2" t="n">
         <v>45862</v>
       </c>
     </row>
@@ -2257,7 +2254,7 @@
       <c r="E70" t="n">
         <v>15.41</v>
       </c>
-      <c r="F70" s="3" t="n">
+      <c r="F70" s="2" t="n">
         <v>45863</v>
       </c>
     </row>
@@ -2283,7 +2280,7 @@
       <c r="E71" t="n">
         <v>15.41</v>
       </c>
-      <c r="F71" s="3" t="n">
+      <c r="F71" s="2" t="n">
         <v>45864</v>
       </c>
     </row>
@@ -2309,7 +2306,7 @@
       <c r="E72" t="n">
         <v>15.41</v>
       </c>
-      <c r="F72" s="3" t="n">
+      <c r="F72" s="2" t="n">
         <v>45865</v>
       </c>
     </row>
@@ -2335,7 +2332,7 @@
       <c r="E73" t="n">
         <v>15.41</v>
       </c>
-      <c r="F73" s="3" t="n">
+      <c r="F73" s="2" t="n">
         <v>45866</v>
       </c>
     </row>
@@ -2361,7 +2358,7 @@
       <c r="E74" t="n">
         <v>14.75</v>
       </c>
-      <c r="F74" s="3" t="n">
+      <c r="F74" s="2" t="n">
         <v>45867</v>
       </c>
     </row>
@@ -2387,7 +2384,7 @@
       <c r="E75" t="n">
         <v>14.75</v>
       </c>
-      <c r="F75" s="3" t="n">
+      <c r="F75" s="2" t="n">
         <v>45868</v>
       </c>
     </row>
@@ -2413,7 +2410,7 @@
       <c r="E76" t="n">
         <v>15.41</v>
       </c>
-      <c r="F76" s="3" t="n">
+      <c r="F76" s="2" t="n">
         <v>45869</v>
       </c>
     </row>
@@ -2439,7 +2436,7 @@
       <c r="E77" t="n">
         <v>15.41</v>
       </c>
-      <c r="F77" s="3" t="n">
+      <c r="F77" s="2" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -2465,7 +2462,7 @@
       <c r="E78" t="n">
         <v>15.41</v>
       </c>
-      <c r="F78" s="3" t="n">
+      <c r="F78" s="2" t="n">
         <v>45871</v>
       </c>
     </row>
@@ -2491,7 +2488,7 @@
       <c r="E79" t="n">
         <v>15.41</v>
       </c>
-      <c r="F79" s="3" t="n">
+      <c r="F79" s="2" t="n">
         <v>45872</v>
       </c>
     </row>
@@ -2517,7 +2514,7 @@
       <c r="E80" t="n">
         <v>14.75</v>
       </c>
-      <c r="F80" s="3" t="n">
+      <c r="F80" s="2" t="n">
         <v>45873</v>
       </c>
     </row>
@@ -2543,7 +2540,7 @@
       <c r="E81" t="n">
         <v>12.88</v>
       </c>
-      <c r="F81" s="3" t="n">
+      <c r="F81" s="2" t="n">
         <v>45874</v>
       </c>
     </row>
@@ -2569,7 +2566,7 @@
       <c r="E82" t="n">
         <v>12.88</v>
       </c>
-      <c r="F82" s="3" t="n">
+      <c r="F82" s="2" t="n">
         <v>45875</v>
       </c>
     </row>
@@ -2595,7 +2592,7 @@
       <c r="E83" t="n">
         <v>12.88</v>
       </c>
-      <c r="F83" s="3" t="n">
+      <c r="F83" s="2" t="n">
         <v>45876</v>
       </c>
     </row>
@@ -2621,7 +2618,7 @@
       <c r="E84" t="n">
         <v>15.41</v>
       </c>
-      <c r="F84" s="3" t="n">
+      <c r="F84" s="2" t="n">
         <v>45877</v>
       </c>
     </row>
@@ -2647,7 +2644,7 @@
       <c r="E85" t="n">
         <v>15.41</v>
       </c>
-      <c r="F85" s="3" t="n">
+      <c r="F85" s="2" t="n">
         <v>45878</v>
       </c>
     </row>
@@ -2673,7 +2670,7 @@
       <c r="E86" t="n">
         <v>15.41</v>
       </c>
-      <c r="F86" s="3" t="n">
+      <c r="F86" s="2" t="n">
         <v>45879</v>
       </c>
     </row>
@@ -2699,7 +2696,7 @@
       <c r="E87" t="n">
         <v>15.41</v>
       </c>
-      <c r="F87" s="3" t="n">
+      <c r="F87" s="2" t="n">
         <v>45880</v>
       </c>
     </row>
@@ -2725,7 +2722,7 @@
       <c r="E88" t="n">
         <v>14.75</v>
       </c>
-      <c r="F88" s="3" t="n">
+      <c r="F88" s="2" t="n">
         <v>45881</v>
       </c>
     </row>
@@ -2751,7 +2748,7 @@
       <c r="E89" t="n">
         <v>14.75</v>
       </c>
-      <c r="F89" s="3" t="n">
+      <c r="F89" s="2" t="n">
         <v>45882</v>
       </c>
     </row>
@@ -2777,7 +2774,7 @@
       <c r="E90" t="n">
         <v>14.75</v>
       </c>
-      <c r="F90" s="3" t="n">
+      <c r="F90" s="2" t="n">
         <v>45883</v>
       </c>
     </row>
@@ -2803,7 +2800,7 @@
       <c r="E91" t="n">
         <v>14.75</v>
       </c>
-      <c r="F91" s="3" t="n">
+      <c r="F91" s="2" t="n">
         <v>45884</v>
       </c>
     </row>
@@ -2829,7 +2826,7 @@
       <c r="E92" t="n">
         <v>15.41</v>
       </c>
-      <c r="F92" s="3" t="n">
+      <c r="F92" s="2" t="n">
         <v>45885</v>
       </c>
     </row>
@@ -2855,7 +2852,7 @@
       <c r="E93" t="n">
         <v>14.75</v>
       </c>
-      <c r="F93" s="3" t="n">
+      <c r="F93" s="2" t="n">
         <v>45886</v>
       </c>
     </row>
@@ -2881,7 +2878,7 @@
       <c r="E94" t="n">
         <v>14.75</v>
       </c>
-      <c r="F94" s="3" t="n">
+      <c r="F94" s="2" t="n">
         <v>45887</v>
       </c>
     </row>
@@ -2907,7 +2904,7 @@
       <c r="E95" t="n">
         <v>14.75</v>
       </c>
-      <c r="F95" s="3" t="n">
+      <c r="F95" s="2" t="n">
         <v>45888</v>
       </c>
     </row>
@@ -2933,7 +2930,7 @@
       <c r="E96" t="n">
         <v>14.75</v>
       </c>
-      <c r="F96" s="3" t="n">
+      <c r="F96" s="2" t="n">
         <v>45889</v>
       </c>
     </row>
@@ -2959,7 +2956,7 @@
       <c r="E97" t="n">
         <v>15.41</v>
       </c>
-      <c r="F97" s="3" t="n">
+      <c r="F97" s="2" t="n">
         <v>45890</v>
       </c>
     </row>
@@ -2985,7 +2982,7 @@
       <c r="E98" t="n">
         <v>14.75</v>
       </c>
-      <c r="F98" s="3" t="n">
+      <c r="F98" s="2" t="n">
         <v>45891</v>
       </c>
     </row>
@@ -3011,7 +3008,7 @@
       <c r="E99" t="n">
         <v>15.41</v>
       </c>
-      <c r="F99" s="3" t="n">
+      <c r="F99" s="2" t="n">
         <v>45892</v>
       </c>
     </row>
@@ -3037,7 +3034,7 @@
       <c r="E100" t="n">
         <v>14.75</v>
       </c>
-      <c r="F100" s="3" t="n">
+      <c r="F100" s="2" t="n">
         <v>45893</v>
       </c>
     </row>
@@ -3063,7 +3060,7 @@
       <c r="E101" t="n">
         <v>15.41</v>
       </c>
-      <c r="F101" s="3" t="n">
+      <c r="F101" s="2" t="n">
         <v>45895</v>
       </c>
     </row>
@@ -3089,7 +3086,7 @@
       <c r="E102" t="n">
         <v>15.41</v>
       </c>
-      <c r="F102" s="3" t="n">
+      <c r="F102" s="2" t="n">
         <v>45896</v>
       </c>
     </row>
@@ -3115,7 +3112,7 @@
       <c r="E103" t="n">
         <v>14</v>
       </c>
-      <c r="F103" s="3" t="n">
+      <c r="F103" s="2" t="n">
         <v>45897</v>
       </c>
     </row>
@@ -3141,7 +3138,7 @@
       <c r="E104" t="n">
         <v>15.41</v>
       </c>
-      <c r="F104" s="3" t="n">
+      <c r="F104" s="2" t="n">
         <v>45898</v>
       </c>
     </row>
@@ -3167,7 +3164,7 @@
       <c r="E105" t="n">
         <v>15.41</v>
       </c>
-      <c r="F105" s="3" t="n">
+      <c r="F105" s="2" t="n">
         <v>45899</v>
       </c>
     </row>
@@ -3193,7 +3190,7 @@
       <c r="E106" t="n">
         <v>14</v>
       </c>
-      <c r="F106" s="3" t="n">
+      <c r="F106" s="2" t="n">
         <v>45900</v>
       </c>
     </row>
@@ -3219,7 +3216,7 @@
       <c r="E107" t="n">
         <v>11.67</v>
       </c>
-      <c r="F107" s="3" t="n">
+      <c r="F107" s="2" t="n">
         <v>45901</v>
       </c>
     </row>
@@ -3245,7 +3242,7 @@
       <c r="E108" t="n">
         <v>14</v>
       </c>
-      <c r="F108" s="3" t="n">
+      <c r="F108" s="2" t="n">
         <v>45902</v>
       </c>
     </row>
@@ -3271,7 +3268,7 @@
       <c r="E109" t="n">
         <v>15.41</v>
       </c>
-      <c r="F109" s="3" t="n">
+      <c r="F109" s="2" t="n">
         <v>45903</v>
       </c>
     </row>
@@ -3297,7 +3294,7 @@
       <c r="E110" t="n">
         <v>15.41</v>
       </c>
-      <c r="F110" s="3" t="n">
+      <c r="F110" s="2" t="n">
         <v>45904</v>
       </c>
     </row>
@@ -3323,7 +3320,7 @@
       <c r="E111" t="n">
         <v>15.41</v>
       </c>
-      <c r="F111" s="3" t="n">
+      <c r="F111" s="2" t="n">
         <v>45905</v>
       </c>
     </row>
@@ -3349,7 +3346,7 @@
       <c r="E112" t="n">
         <v>15.41</v>
       </c>
-      <c r="F112" s="3" t="n">
+      <c r="F112" s="2" t="n">
         <v>45906</v>
       </c>
     </row>
@@ -3375,7 +3372,7 @@
       <c r="E113" t="n">
         <v>14</v>
       </c>
-      <c r="F113" s="3" t="n">
+      <c r="F113" s="2" t="n">
         <v>45907</v>
       </c>
     </row>
@@ -3401,7 +3398,7 @@
       <c r="E114" t="n">
         <v>15.41</v>
       </c>
-      <c r="F114" s="3" t="n">
+      <c r="F114" s="2" t="n">
         <v>45908</v>
       </c>
     </row>
@@ -3427,7 +3424,7 @@
       <c r="E115" t="n">
         <v>11.67</v>
       </c>
-      <c r="F115" s="3" t="n">
+      <c r="F115" s="2" t="n">
         <v>45909</v>
       </c>
     </row>
@@ -3453,7 +3450,7 @@
       <c r="E116" t="n">
         <v>15.41</v>
       </c>
-      <c r="F116" s="3" t="n">
+      <c r="F116" s="2" t="n">
         <v>45910</v>
       </c>
     </row>
@@ -3479,7 +3476,7 @@
       <c r="E117" t="n">
         <v>11.67</v>
       </c>
-      <c r="F117" s="3" t="n">
+      <c r="F117" s="2" t="n">
         <v>45911</v>
       </c>
     </row>
@@ -3505,7 +3502,7 @@
       <c r="E118" t="n">
         <v>15.41</v>
       </c>
-      <c r="F118" s="3" t="n">
+      <c r="F118" s="2" t="n">
         <v>45912</v>
       </c>
     </row>
@@ -3531,7 +3528,7 @@
       <c r="E119" t="n">
         <v>15.41</v>
       </c>
-      <c r="F119" s="3" t="n">
+      <c r="F119" s="2" t="n">
         <v>45913</v>
       </c>
     </row>
@@ -3557,7 +3554,7 @@
       <c r="E120" t="n">
         <v>15.41</v>
       </c>
-      <c r="F120" s="3" t="n">
+      <c r="F120" s="2" t="n">
         <v>45914</v>
       </c>
     </row>
@@ -3583,7 +3580,7 @@
       <c r="E121" t="n">
         <v>14.75</v>
       </c>
-      <c r="F121" s="3" t="n">
+      <c r="F121" s="2" t="n">
         <v>45915</v>
       </c>
     </row>
@@ -3609,7 +3606,7 @@
       <c r="E122" t="n">
         <v>11.67</v>
       </c>
-      <c r="F122" s="3" t="n">
+      <c r="F122" s="2" t="n">
         <v>45916</v>
       </c>
     </row>
@@ -3635,7 +3632,7 @@
       <c r="E123" t="n">
         <v>11.67</v>
       </c>
-      <c r="F123" s="3" t="n">
+      <c r="F123" s="2" t="n">
         <v>45917</v>
       </c>
     </row>
@@ -3661,7 +3658,7 @@
       <c r="E124" t="n">
         <v>14</v>
       </c>
-      <c r="F124" s="3" t="n">
+      <c r="F124" s="2" t="n">
         <v>45922</v>
       </c>
     </row>
@@ -3687,7 +3684,7 @@
       <c r="E125" t="n">
         <v>15.41</v>
       </c>
-      <c r="F125" s="3" t="n">
+      <c r="F125" s="2" t="n">
         <v>45923</v>
       </c>
     </row>
@@ -3713,7 +3710,7 @@
       <c r="E126" t="n">
         <v>11.67</v>
       </c>
-      <c r="F126" s="3" t="n">
+      <c r="F126" s="2" t="n">
         <v>45924</v>
       </c>
     </row>
@@ -3739,7 +3736,7 @@
       <c r="E127" t="n">
         <v>15.41</v>
       </c>
-      <c r="F127" s="3" t="n">
+      <c r="F127" s="2" t="n">
         <v>45925</v>
       </c>
     </row>
@@ -3765,7 +3762,7 @@
       <c r="E128" t="n">
         <v>15.41</v>
       </c>
-      <c r="F128" s="3" t="n">
+      <c r="F128" s="2" t="n">
         <v>45926</v>
       </c>
     </row>
@@ -3791,7 +3788,7 @@
       <c r="E129" t="n">
         <v>15.41</v>
       </c>
-      <c r="F129" s="3" t="n">
+      <c r="F129" s="2" t="n">
         <v>45927</v>
       </c>
     </row>
@@ -3817,7 +3814,7 @@
       <c r="E130" t="n">
         <v>14</v>
       </c>
-      <c r="F130" s="3" t="n">
+      <c r="F130" s="2" t="n">
         <v>45928</v>
       </c>
     </row>
@@ -3843,7 +3840,7 @@
       <c r="E131" t="n">
         <v>11.67</v>
       </c>
-      <c r="F131" s="3" t="n">
+      <c r="F131" s="2" t="n">
         <v>45929</v>
       </c>
     </row>
@@ -3869,7 +3866,7 @@
       <c r="E132" t="n">
         <v>15.41</v>
       </c>
-      <c r="F132" s="3" t="n">
+      <c r="F132" s="2" t="n">
         <v>45930</v>
       </c>
     </row>
@@ -3895,7 +3892,7 @@
       <c r="E133" t="n">
         <v>11.67</v>
       </c>
-      <c r="F133" s="3" t="n">
+      <c r="F133" s="2" t="n">
         <v>45931</v>
       </c>
     </row>
@@ -3921,7 +3918,7 @@
       <c r="E134" t="n">
         <v>15.41</v>
       </c>
-      <c r="F134" s="3" t="n">
+      <c r="F134" s="2" t="n">
         <v>45932</v>
       </c>
     </row>
@@ -3947,7 +3944,7 @@
       <c r="E135" t="n">
         <v>11.67</v>
       </c>
-      <c r="F135" s="3" t="n">
+      <c r="F135" s="2" t="n">
         <v>45933</v>
       </c>
     </row>
@@ -3973,7 +3970,7 @@
       <c r="E136" t="n">
         <v>15.41</v>
       </c>
-      <c r="F136" s="3" t="n">
+      <c r="F136" s="2" t="n">
         <v>45934</v>
       </c>
     </row>
@@ -3999,7 +3996,7 @@
       <c r="E137" t="n">
         <v>15.41</v>
       </c>
-      <c r="F137" s="3" t="n">
+      <c r="F137" s="2" t="n">
         <v>45935</v>
       </c>
     </row>
@@ -4025,7 +4022,7 @@
       <c r="E138" t="n">
         <v>11.67</v>
       </c>
-      <c r="F138" s="3" t="n">
+      <c r="F138" s="2" t="n">
         <v>45936</v>
       </c>
     </row>
@@ -4051,7 +4048,7 @@
       <c r="E139" t="n">
         <v>15.41</v>
       </c>
-      <c r="F139" s="3" t="n">
+      <c r="F139" s="2" t="n">
         <v>45937</v>
       </c>
     </row>
@@ -4077,7 +4074,7 @@
       <c r="E140" t="n">
         <v>11.67</v>
       </c>
-      <c r="F140" s="3" t="n">
+      <c r="F140" s="2" t="n">
         <v>45938</v>
       </c>
     </row>
@@ -4103,7 +4100,7 @@
       <c r="E141" t="n">
         <v>15.41</v>
       </c>
-      <c r="F141" s="3" t="n">
+      <c r="F141" s="2" t="n">
         <v>45939</v>
       </c>
     </row>
@@ -4129,7 +4126,7 @@
       <c r="E142" t="n">
         <v>14</v>
       </c>
-      <c r="F142" s="3" t="n">
+      <c r="F142" s="2" t="n">
         <v>45940</v>
       </c>
     </row>
@@ -4155,7 +4152,7 @@
       <c r="E143" t="n">
         <v>15.41</v>
       </c>
-      <c r="F143" s="3" t="n">
+      <c r="F143" s="2" t="n">
         <v>45941</v>
       </c>
     </row>
@@ -4181,7 +4178,7 @@
       <c r="E144" t="n">
         <v>14</v>
       </c>
-      <c r="F144" s="3" t="n">
+      <c r="F144" s="2" t="n">
         <v>45942</v>
       </c>
     </row>
@@ -4207,7 +4204,7 @@
       <c r="E145" t="n">
         <v>14</v>
       </c>
-      <c r="F145" s="3" t="n">
+      <c r="F145" s="2" t="n">
         <v>45943</v>
       </c>
     </row>
@@ -4233,7 +4230,7 @@
       <c r="E146" t="n">
         <v>14</v>
       </c>
-      <c r="F146" s="3" t="n">
+      <c r="F146" s="2" t="n">
         <v>45944</v>
       </c>
     </row>
@@ -4259,7 +4256,7 @@
       <c r="E147" t="n">
         <v>14</v>
       </c>
-      <c r="F147" s="3" t="n">
+      <c r="F147" s="2" t="n">
         <v>45945</v>
       </c>
     </row>
@@ -4285,7 +4282,7 @@
       <c r="E148" t="n">
         <v>14</v>
       </c>
-      <c r="F148" s="3" t="n">
+      <c r="F148" s="2" t="n">
         <v>45946</v>
       </c>
     </row>
@@ -4311,7 +4308,7 @@
       <c r="E149" t="n">
         <v>14</v>
       </c>
-      <c r="F149" s="3" t="n">
+      <c r="F149" s="2" t="n">
         <v>45947</v>
       </c>
     </row>
@@ -4337,7 +4334,7 @@
       <c r="E150" t="n">
         <v>14</v>
       </c>
-      <c r="F150" s="3" t="n">
+      <c r="F150" s="2" t="n">
         <v>45950</v>
       </c>
     </row>
@@ -4363,7 +4360,7 @@
       <c r="E151" t="n">
         <v>14</v>
       </c>
-      <c r="F151" s="3" t="n">
+      <c r="F151" s="2" t="n">
         <v>45951</v>
       </c>
     </row>
@@ -4389,7 +4386,7 @@
       <c r="E152" t="n">
         <v>15.41</v>
       </c>
-      <c r="F152" s="3" t="n">
+      <c r="F152" s="2" t="n">
         <v>45952</v>
       </c>
     </row>
@@ -4415,7 +4412,7 @@
       <c r="E153" t="n">
         <v>14</v>
       </c>
-      <c r="F153" s="3" t="n">
+      <c r="F153" s="2" t="n">
         <v>45953</v>
       </c>
     </row>
@@ -4441,7 +4438,7 @@
       <c r="E154" t="n">
         <v>14</v>
       </c>
-      <c r="F154" s="3" t="n">
+      <c r="F154" s="2" t="n">
         <v>45954</v>
       </c>
     </row>
@@ -4467,7 +4464,7 @@
       <c r="E155" t="n">
         <v>15.41</v>
       </c>
-      <c r="F155" s="3" t="n">
+      <c r="F155" s="2" t="n">
         <v>45955</v>
       </c>
     </row>
@@ -4493,7 +4490,7 @@
       <c r="E156" t="n">
         <v>14</v>
       </c>
-      <c r="F156" s="3" t="n">
+      <c r="F156" s="2" t="n">
         <v>45956</v>
       </c>
     </row>
@@ -4519,7 +4516,7 @@
       <c r="E157" t="n">
         <v>14</v>
       </c>
-      <c r="F157" s="3" t="n">
+      <c r="F157" s="2" t="n">
         <v>45957</v>
       </c>
     </row>
@@ -4545,7 +4542,7 @@
       <c r="E158" t="n">
         <v>14</v>
       </c>
-      <c r="F158" s="3" t="n">
+      <c r="F158" s="2" t="n">
         <v>45958</v>
       </c>
     </row>
@@ -4571,7 +4568,7 @@
       <c r="E159" t="n">
         <v>14</v>
       </c>
-      <c r="F159" s="3" t="n">
+      <c r="F159" s="2" t="n">
         <v>45958</v>
       </c>
     </row>
@@ -4597,7 +4594,7 @@
       <c r="E160" t="n">
         <v>14</v>
       </c>
-      <c r="F160" s="3" t="n">
+      <c r="F160" s="2" t="n">
         <v>45958</v>
       </c>
     </row>
@@ -4623,7 +4620,7 @@
       <c r="E161" t="n">
         <v>14</v>
       </c>
-      <c r="F161" s="3" t="n">
+      <c r="F161" s="2" t="n">
         <v>45964</v>
       </c>
     </row>
@@ -4649,7 +4646,7 @@
       <c r="E162" t="n">
         <v>14</v>
       </c>
-      <c r="F162" s="3" t="n">
+      <c r="F162" s="2" t="n">
         <v>45966</v>
       </c>
     </row>
@@ -4675,7 +4672,7 @@
       <c r="E163" t="n">
         <v>14</v>
       </c>
-      <c r="F163" s="3" t="n">
+      <c r="F163" s="2" t="n">
         <v>45966</v>
       </c>
     </row>
@@ -4701,7 +4698,7 @@
       <c r="E164" t="n">
         <v>14</v>
       </c>
-      <c r="F164" s="3" t="n">
+      <c r="F164" s="2" t="n">
         <v>45966</v>
       </c>
     </row>
@@ -4727,7 +4724,7 @@
       <c r="E165" t="n">
         <v>14</v>
       </c>
-      <c r="F165" s="3" t="n">
+      <c r="F165" s="2" t="n">
         <v>45967</v>
       </c>
     </row>
@@ -4753,7 +4750,7 @@
       <c r="E166" t="n">
         <v>15.41</v>
       </c>
-      <c r="F166" s="3" t="n">
+      <c r="F166" s="2" t="n">
         <v>45968</v>
       </c>
     </row>
@@ -4779,7 +4776,7 @@
       <c r="E167" t="n">
         <v>15.41</v>
       </c>
-      <c r="F167" s="3" t="n">
+      <c r="F167" s="2" t="n">
         <v>45969</v>
       </c>
     </row>
@@ -4805,7 +4802,7 @@
       <c r="E168" t="n">
         <v>14</v>
       </c>
-      <c r="F168" s="3" t="n">
+      <c r="F168" s="2" t="n">
         <v>45970</v>
       </c>
     </row>
@@ -4831,7 +4828,7 @@
       <c r="E169" t="n">
         <v>14</v>
       </c>
-      <c r="F169" s="3" t="n">
+      <c r="F169" s="2" t="n">
         <v>45971</v>
       </c>
     </row>
@@ -4857,7 +4854,7 @@
       <c r="E170" t="n">
         <v>14</v>
       </c>
-      <c r="F170" s="3" t="n">
+      <c r="F170" s="2" t="n">
         <v>45972</v>
       </c>
     </row>
@@ -4883,7 +4880,7 @@
       <c r="E171" t="n">
         <v>15.41</v>
       </c>
-      <c r="F171" s="3" t="n">
+      <c r="F171" s="2" t="n">
         <v>45973</v>
       </c>
     </row>
@@ -4909,7 +4906,7 @@
       <c r="E172" t="n">
         <v>14</v>
       </c>
-      <c r="F172" s="3" t="n">
+      <c r="F172" s="2" t="n">
         <v>45974</v>
       </c>
     </row>
@@ -4935,7 +4932,7 @@
       <c r="E173" t="n">
         <v>14</v>
       </c>
-      <c r="F173" s="3" t="n">
+      <c r="F173" s="2" t="n">
         <v>45978</v>
       </c>
     </row>
@@ -4961,7 +4958,7 @@
       <c r="E174" t="n">
         <v>14</v>
       </c>
-      <c r="F174" s="3" t="n">
+      <c r="F174" s="2" t="n">
         <v>45979</v>
       </c>
     </row>
@@ -4987,7 +4984,7 @@
       <c r="E175" t="n">
         <v>15.41</v>
       </c>
-      <c r="F175" s="3" t="n">
+      <c r="F175" s="2" t="n">
         <v>45980</v>
       </c>
     </row>
@@ -5013,7 +5010,7 @@
       <c r="E176" t="n">
         <v>14</v>
       </c>
-      <c r="F176" s="3" t="n">
+      <c r="F176" s="2" t="n">
         <v>45981</v>
       </c>
     </row>
@@ -5039,7 +5036,7 @@
       <c r="E177" t="n">
         <v>10.9</v>
       </c>
-      <c r="F177" s="3" t="n">
+      <c r="F177" s="2" t="n">
         <v>45985</v>
       </c>
     </row>
@@ -5065,7 +5062,7 @@
       <c r="E178" t="n">
         <v>10.9</v>
       </c>
-      <c r="F178" s="3" t="n">
+      <c r="F178" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5091,7 +5088,7 @@
       <c r="E179" t="n">
         <v>10.9</v>
       </c>
-      <c r="F179" s="3" t="n">
+      <c r="F179" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5117,7 +5114,7 @@
       <c r="E180" t="n">
         <v>10.9</v>
       </c>
-      <c r="F180" s="3" t="n">
+      <c r="F180" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5143,7 +5140,7 @@
       <c r="E181" t="n">
         <v>10.9</v>
       </c>
-      <c r="F181" s="3" t="n">
+      <c r="F181" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5169,7 +5166,7 @@
       <c r="E182" t="n">
         <v>10.9</v>
       </c>
-      <c r="F182" s="3" t="n">
+      <c r="F182" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5195,7 +5192,7 @@
       <c r="E183" t="n">
         <v>10.9</v>
       </c>
-      <c r="F183" s="3" t="n">
+      <c r="F183" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5221,7 +5218,7 @@
       <c r="E184" t="n">
         <v>10.9</v>
       </c>
-      <c r="F184" s="3" t="n">
+      <c r="F184" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5247,7 +5244,7 @@
       <c r="E185" t="n">
         <v>10.9</v>
       </c>
-      <c r="F185" s="3" t="n">
+      <c r="F185" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5273,7 +5270,7 @@
       <c r="E186" t="n">
         <v>10.9</v>
       </c>
-      <c r="F186" s="3" t="n">
+      <c r="F186" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5299,7 +5296,7 @@
       <c r="E187" t="n">
         <v>10.9</v>
       </c>
-      <c r="F187" s="3" t="n">
+      <c r="F187" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5325,7 +5322,7 @@
       <c r="E188" t="n">
         <v>10.9</v>
       </c>
-      <c r="F188" s="3" t="n">
+      <c r="F188" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5351,7 +5348,7 @@
       <c r="E189" t="n">
         <v>10.9</v>
       </c>
-      <c r="F189" s="3" t="n">
+      <c r="F189" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5377,7 +5374,7 @@
       <c r="E190" t="n">
         <v>10.9</v>
       </c>
-      <c r="F190" s="3" t="n">
+      <c r="F190" s="2" t="n">
         <v>45986</v>
       </c>
     </row>
@@ -5403,7 +5400,7 @@
       <c r="E191" t="n">
         <v>10.9</v>
       </c>
-      <c r="F191" s="3" t="n">
+      <c r="F191" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5429,7 +5426,7 @@
       <c r="E192" t="n">
         <v>10.9</v>
       </c>
-      <c r="F192" s="3" t="n">
+      <c r="F192" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5455,7 +5452,7 @@
       <c r="E193" t="n">
         <v>10.9</v>
       </c>
-      <c r="F193" s="3" t="n">
+      <c r="F193" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5481,7 +5478,7 @@
       <c r="E194" t="n">
         <v>10.9</v>
       </c>
-      <c r="F194" s="3" t="n">
+      <c r="F194" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5507,7 +5504,7 @@
       <c r="E195" t="n">
         <v>10.9</v>
       </c>
-      <c r="F195" s="3" t="n">
+      <c r="F195" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5533,7 +5530,7 @@
       <c r="E196" t="n">
         <v>10.9</v>
       </c>
-      <c r="F196" s="3" t="n">
+      <c r="F196" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5559,7 +5556,7 @@
       <c r="E197" t="n">
         <v>10.9</v>
       </c>
-      <c r="F197" s="3" t="n">
+      <c r="F197" s="2" t="n">
         <v>45987</v>
       </c>
     </row>
@@ -5585,7 +5582,7 @@
       <c r="E198" t="n">
         <v>22.5</v>
       </c>
-      <c r="F198" s="3" t="n">
+      <c r="F198" s="2" t="n">
         <v>46144</v>
       </c>
     </row>
@@ -5611,7 +5608,7 @@
       <c r="E199" t="n">
         <v>22.5</v>
       </c>
-      <c r="F199" s="3" t="n">
+      <c r="F199" s="2" t="n">
         <v>46144</v>
       </c>
     </row>
@@ -5637,13 +5634,13 @@
       <c r="E200" t="n">
         <v>22.5</v>
       </c>
-      <c r="F200" s="3" t="n">
+      <c r="F200" s="2" t="n">
         <v>46144</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
-        <v>46144.71269611372</v>
+        <v>46144.71269611111</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -5662,6 +5659,28 @@
       </c>
       <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46245.69201655036</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>20,45 €</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mejora formulario de actualización manual de precios
</commit_message>
<xml_diff>
--- a/data/precios_creatina.xlsx
+++ b/data/precios_creatina.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F202"/>
+  <dimension ref="A1:F208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5662,7 +5662,7 @@
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
-        <v>46245.69201655036</v>
+        <v>46245.69201655093</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -5681,6 +5681,138 @@
       </c>
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46246.40221082176</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>14,00 €</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46247.40486728009</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>20,45 €</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46248.39678311343</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>14,00 €</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>46251.39828439815</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>14,00 €</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>46252.40829810185</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>14,00 €</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>46253.48337625423</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>1Kg</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>14,00 €</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>